<commit_message>
evaluation of outputs: format + llm_as_judge + facts check
</commit_message>
<xml_diff>
--- a/examples/comps.xlsx
+++ b/examples/comps.xlsx
@@ -292,82 +292,82 @@
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
       <text>
+        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
+      </text>
+    </comment>
+    <comment ref="C13" authorId="0" shapeId="0">
+      <text>
+        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
+      </text>
+    </comment>
+    <comment ref="D13" authorId="0" shapeId="0">
+      <text>
+        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
+      </text>
+    </comment>
+    <comment ref="E13" authorId="0" shapeId="0">
+      <text>
+        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
         <t>Source: Yahoo Finance (DUK), retrieved via yfinance</t>
       </text>
     </comment>
-    <comment ref="C13" authorId="0" shapeId="0">
+    <comment ref="C14" authorId="0" shapeId="0">
       <text>
         <t>Source: Yahoo Finance (DUK), retrieved via yfinance</t>
       </text>
     </comment>
-    <comment ref="D13" authorId="0" shapeId="0">
+    <comment ref="D14" authorId="0" shapeId="0">
       <text>
         <t>Source: Yahoo Finance (DUK), retrieved via yfinance</t>
       </text>
     </comment>
-    <comment ref="E13" authorId="0" shapeId="0">
+    <comment ref="E14" authorId="0" shapeId="0">
       <text>
         <t>Source: Yahoo Finance (DUK), retrieved via yfinance</t>
       </text>
     </comment>
-    <comment ref="B14" authorId="0" shapeId="0">
+    <comment ref="B15" authorId="0" shapeId="0">
       <text>
         <t>Source: Yahoo Finance (SO), retrieved via yfinance</t>
       </text>
     </comment>
-    <comment ref="C14" authorId="0" shapeId="0">
+    <comment ref="C15" authorId="0" shapeId="0">
       <text>
         <t>Source: Yahoo Finance (SO), retrieved via yfinance</t>
       </text>
     </comment>
-    <comment ref="D14" authorId="0" shapeId="0">
+    <comment ref="D15" authorId="0" shapeId="0">
       <text>
         <t>Source: Yahoo Finance (SO), retrieved via yfinance</t>
       </text>
     </comment>
-    <comment ref="E14" authorId="0" shapeId="0">
+    <comment ref="E15" authorId="0" shapeId="0">
       <text>
         <t>Source: Yahoo Finance (SO), retrieved via yfinance</t>
       </text>
     </comment>
-    <comment ref="B15" authorId="0" shapeId="0">
-      <text>
-        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
-      </text>
-    </comment>
-    <comment ref="C15" authorId="0" shapeId="0">
-      <text>
-        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
-      </text>
-    </comment>
-    <comment ref="D15" authorId="0" shapeId="0">
-      <text>
-        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
-      </text>
-    </comment>
-    <comment ref="E15" authorId="0" shapeId="0">
-      <text>
-        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
-      </text>
-    </comment>
     <comment ref="B16" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (GEV), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (AWK), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C16" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (GEV), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (AWK), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D16" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (GEV), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (AWK), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E16" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (GEV), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (AWK), retrieved via yfinance</t>
       </text>
     </comment>
   </commentList>
@@ -724,13 +724,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71060</v>
+        <v>68470</v>
       </c>
       <c r="C5" t="n">
         <v>6790</v>
       </c>
       <c r="D5" t="n">
-        <v>146.22</v>
+        <v>146.38</v>
       </c>
       <c r="E5" t="n">
         <v>5.98</v>
@@ -751,16 +751,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>112832</v>
+        <v>111048</v>
       </c>
       <c r="C6" t="n">
         <v>7957</v>
       </c>
       <c r="D6" t="n">
-        <v>251.65</v>
+        <v>246.71</v>
       </c>
       <c r="E6" t="n">
-        <v>11.5</v>
+        <v>11.51</v>
       </c>
       <c r="F6">
         <f>B6/C6</f>
@@ -778,16 +778,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>51250</v>
+        <v>49929</v>
       </c>
       <c r="C7" t="n">
         <v>2258</v>
       </c>
       <c r="D7" t="n">
-        <v>129.96</v>
+        <v>123.7</v>
       </c>
       <c r="E7" t="n">
-        <v>0.91</v>
+        <v>0.9</v>
       </c>
       <c r="F7">
         <f>B7/C7</f>
@@ -805,16 +805,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>81003</v>
+        <v>81378</v>
       </c>
       <c r="C8" t="n">
         <v>5490.2</v>
       </c>
       <c r="D8" t="n">
-        <v>109.66</v>
+        <v>109.89</v>
       </c>
       <c r="E8" t="n">
-        <v>3.91</v>
+        <v>3.92</v>
       </c>
       <c r="F8">
         <f>B8/C8</f>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>96910</v>
+        <v>97197</v>
       </c>
       <c r="C9" t="n">
         <v>8249</v>
       </c>
       <c r="D9" t="n">
-        <v>45.33</v>
+        <v>45.51</v>
       </c>
       <c r="E9" t="n">
         <v>2.73</v>
@@ -859,13 +859,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>48439</v>
+        <v>48446</v>
       </c>
       <c r="C10" t="n">
         <v>3755</v>
       </c>
       <c r="D10" t="n">
-        <v>14.66</v>
+        <v>14.67</v>
       </c>
       <c r="E10" t="n">
         <v>1.92</v>
@@ -886,13 +886,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>100154</v>
+        <v>100616</v>
       </c>
       <c r="C11" t="n">
         <v>10313</v>
       </c>
       <c r="D11" t="n">
-        <v>16.58</v>
+        <v>16.79</v>
       </c>
       <c r="E11" t="n">
         <v>1.29</v>
@@ -913,16 +913,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>56016</v>
+        <v>56455</v>
       </c>
       <c r="C12" t="n">
         <v>5170</v>
       </c>
       <c r="D12" t="n">
-        <v>45.91</v>
+        <v>46.67</v>
       </c>
       <c r="E12" t="n">
-        <v>1.85</v>
+        <v>1.84</v>
       </c>
       <c r="F12">
         <f>B12/C12</f>
@@ -936,20 +936,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>188593</v>
+        <v>290735</v>
       </c>
       <c r="C13" t="n">
-        <v>16478</v>
+        <v>14159</v>
       </c>
       <c r="D13" t="n">
-        <v>123.82</v>
+        <v>84.84</v>
       </c>
       <c r="E13" t="n">
-        <v>6.5</v>
+        <v>3.94</v>
       </c>
       <c r="F13">
         <f>B13/C13</f>
@@ -963,20 +963,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>182597</v>
+        <v>188881</v>
       </c>
       <c r="C14" t="n">
-        <v>13974</v>
+        <v>16478</v>
       </c>
       <c r="D14" t="n">
-        <v>92.95</v>
+        <v>124.19</v>
       </c>
       <c r="E14" t="n">
-        <v>3.91</v>
+        <v>6.5</v>
       </c>
       <c r="F14">
         <f>B14/C14</f>
@@ -990,20 +990,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>290715</v>
+        <v>182957</v>
       </c>
       <c r="C15" t="n">
-        <v>14159</v>
+        <v>13974</v>
       </c>
       <c r="D15" t="n">
-        <v>84.83</v>
+        <v>93.27</v>
       </c>
       <c r="E15" t="n">
-        <v>3.94</v>
+        <v>3.91</v>
       </c>
       <c r="F15">
         <f>B15/C15</f>
@@ -1017,20 +1017,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>AWK</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>242389</v>
+        <v>39829</v>
       </c>
       <c r="C16" t="n">
-        <v>3415</v>
+        <v>2836</v>
       </c>
       <c r="D16" t="n">
-        <v>920.15</v>
+        <v>124.45</v>
       </c>
       <c r="E16" t="n">
-        <v>34.23</v>
+        <v>5.64</v>
       </c>
       <c r="F16">
         <f>B16/C16</f>

</xml_diff>

<commit_message>
add benchmark sample outputs: 20-sector primers
</commit_message>
<xml_diff>
--- a/examples/comps.xlsx
+++ b/examples/comps.xlsx
@@ -132,242 +132,242 @@
   <commentList>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (VST), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (EQIX), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C5" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (VST), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (EQIX), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D5" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (VST), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (EQIX), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E5" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (VST), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (EQIX), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (CEG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (DLR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C6" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (CEG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (DLR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D6" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (CEG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (DLR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E6" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (CEG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (DLR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B7" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (NRG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (IRM), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C7" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (NRG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (IRM), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D7" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (NRG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (IRM), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E7" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (NRG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (IRM), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B8" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (ETR), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (CONE), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C8" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (ETR), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (CONE), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D8" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (ETR), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (CONE), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E8" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (ETR), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (CONE), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B9" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (EXC), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (QTS), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C9" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (EXC), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (QTS), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D9" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (EXC), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (QTS), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E9" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (EXC), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (QTS), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B10" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (AES), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (COR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C10" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (AES), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (COR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D10" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (AES), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (COR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E10" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (AES), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (COR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B11" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (PCG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (SWCH), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C11" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (PCG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (SWCH), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D11" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (PCG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (SWCH), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E11" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (PCG), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (SWCH), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B12" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (FE), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (VRT), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C12" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (FE), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (VRT), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D12" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (FE), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (VRT), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E12" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (FE), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (VRT), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (IRTC), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C13" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (IRTC), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D13" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (IRTC), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E13" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (NEE), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (IRTC), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B14" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (DUK), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (AMT), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C14" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (DUK), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (AMT), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D14" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (DUK), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (AMT), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E14" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (DUK), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (AMT), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B15" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (SO), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (SBAC), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C15" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (SO), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (SBAC), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D15" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (SO), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (SBAC), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E15" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (SO), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (SBAC), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="B16" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (AWK), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (DLR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="C16" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (AWK), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (DLR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="D16" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (AWK), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (DLR), retrieved via yfinance</t>
       </text>
     </comment>
     <comment ref="E16" authorId="0" shapeId="0">
       <text>
-        <t>Source: Yahoo Finance (AWK), retrieved via yfinance</t>
+        <t>Source: Yahoo Finance (DLR), retrieved via yfinance</t>
       </text>
     </comment>
   </commentList>
@@ -669,7 +669,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>US DATA-CENTER POWER — COMPARABLE COMPANY ANALYSIS</t>
+          <t>US DATA CENTER REITS — COMPARABLE COMPANY ANALYSIS</t>
         </is>
       </c>
     </row>
@@ -720,20 +720,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>68470</v>
+        <v>122849</v>
       </c>
       <c r="C5" t="n">
-        <v>6790</v>
+        <v>4282</v>
       </c>
       <c r="D5" t="n">
-        <v>146.38</v>
+        <v>1022.6</v>
       </c>
       <c r="E5" t="n">
-        <v>5.98</v>
+        <v>14.43</v>
       </c>
       <c r="F5">
         <f>B5/C5</f>
@@ -747,20 +747,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>111048</v>
+        <v>81620</v>
       </c>
       <c r="C6" t="n">
-        <v>7957</v>
+        <v>2888.7</v>
       </c>
       <c r="D6" t="n">
-        <v>246.71</v>
+        <v>176.07</v>
       </c>
       <c r="E6" t="n">
-        <v>11.51</v>
+        <v>3.84</v>
       </c>
       <c r="F6">
         <f>B6/C6</f>
@@ -774,20 +774,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>49929</v>
+        <v>56557</v>
       </c>
       <c r="C7" t="n">
-        <v>2258</v>
+        <v>2449.7</v>
       </c>
       <c r="D7" t="n">
-        <v>123.7</v>
+        <v>123.52</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9</v>
+        <v>0.93</v>
       </c>
       <c r="F7">
         <f>B7/C7</f>
@@ -801,20 +801,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ETR</t>
+          <t>CONE</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>81378</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>5490.2</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>109.89</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>3.92</v>
+        <v>0</v>
       </c>
       <c r="F8">
         <f>B8/C8</f>
@@ -828,20 +828,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>QTS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>97197</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>8249</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>45.51</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>2.73</v>
+        <v>0</v>
       </c>
       <c r="F9">
         <f>B9/C9</f>
@@ -855,20 +855,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AES</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>48446</v>
+        <v>70804</v>
       </c>
       <c r="C10" t="n">
-        <v>3755</v>
+        <v>5300.4</v>
       </c>
       <c r="D10" t="n">
-        <v>14.67</v>
+        <v>296.57</v>
       </c>
       <c r="E10" t="n">
-        <v>1.92</v>
+        <v>12.81</v>
       </c>
       <c r="F10">
         <f>B10/C10</f>
@@ -882,20 +882,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PCG</t>
+          <t>SWCH</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>100616</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>10313</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>16.79</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>1.29</v>
+        <v>0</v>
       </c>
       <c r="F11">
         <f>B11/C11</f>
@@ -909,20 +909,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>56455</v>
+        <v>117752</v>
       </c>
       <c r="C12" t="n">
-        <v>5170</v>
+        <v>2383</v>
       </c>
       <c r="D12" t="n">
-        <v>46.67</v>
+        <v>304.57</v>
       </c>
       <c r="E12" t="n">
-        <v>1.84</v>
+        <v>3.99</v>
       </c>
       <c r="F12">
         <f>B12/C12</f>
@@ -936,20 +936,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>IRTC</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>290735</v>
+        <v>3902</v>
       </c>
       <c r="C13" t="n">
-        <v>14159</v>
+        <v>-11.2</v>
       </c>
       <c r="D13" t="n">
-        <v>84.84</v>
+        <v>113.26</v>
       </c>
       <c r="E13" t="n">
-        <v>3.94</v>
+        <v>-0.86</v>
       </c>
       <c r="F13">
         <f>B13/C13</f>
@@ -963,20 +963,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>AMT</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>188881</v>
+        <v>128715</v>
       </c>
       <c r="C14" t="n">
-        <v>16478</v>
+        <v>6989.6</v>
       </c>
       <c r="D14" t="n">
-        <v>124.19</v>
+        <v>168.63</v>
       </c>
       <c r="E14" t="n">
-        <v>6.5</v>
+        <v>6.19</v>
       </c>
       <c r="F14">
         <f>B14/C14</f>
@@ -990,20 +990,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>SBAC</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>182957</v>
+        <v>35081</v>
       </c>
       <c r="C15" t="n">
-        <v>13974</v>
+        <v>1827.7</v>
       </c>
       <c r="D15" t="n">
-        <v>93.27</v>
+        <v>187.09</v>
       </c>
       <c r="E15" t="n">
-        <v>3.91</v>
+        <v>9.49</v>
       </c>
       <c r="F15">
         <f>B15/C15</f>
@@ -1017,20 +1017,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AWK</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>39829</v>
+        <v>81620</v>
       </c>
       <c r="C16" t="n">
-        <v>2836</v>
+        <v>2888.7</v>
       </c>
       <c r="D16" t="n">
-        <v>124.45</v>
+        <v>176.07</v>
       </c>
       <c r="E16" t="n">
-        <v>5.64</v>
+        <v>3.84</v>
       </c>
       <c r="F16">
         <f>B16/C16</f>

</xml_diff>